<commit_message>
Added Linnansaari kayak trip.
</commit_message>
<xml_diff>
--- a/data/parks.xlsx
+++ b/data/parks.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentuef-my.sharepoint.com/personal/petrusn_uef_fi/Documents/3_fun_code/vaellus/finnish-national-parks/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{378AD10D-A084-4049-B39D-923DF47C7264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1F2D1A9-8EE7-4A45-B9C8-0CFBD45DECCB}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{378AD10D-A084-4049-B39D-923DF47C7264}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6626634-B043-4734-89DE-5416D3D03CC4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3825" yWindow="4200" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="238">
   <si>
     <t>Etelä-Konneveden kansallispuisto</t>
   </si>
@@ -747,6 +747,9 @@
   </si>
   <si>
     <t>8/2023, 8/2024</t>
+  </si>
+  <si>
+    <t>6/2026</t>
   </si>
 </sst>
 </file>
@@ -1676,7 +1679,10 @@
         <v>130</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>132</v>
+        <v>133</v>
+      </c>
+      <c r="K16" s="11" t="s">
+        <v>237</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -2664,4 +2670,10 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{eef6c6f4-1517-4d56-ab52-17a9868743d2}" enabled="1" method="Privileged" siteId="{87879f2e-7304-4bf2-baf2-63e7f83f3c34}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>